<commit_message>
Use ContAgil SELIC factors for yearly fiscal impact
Default mode now capitalizes subsidies with ContAgil rules (STP col E or
Bacen SGS 11, from day after installment to 30/06/2026). Regenerates the
sample yearly summary under that methodology.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/impacto_fiscal_por_ano.xlsx
+++ b/output/impacto_fiscal_por_ano.xlsx
@@ -443,13 +443,13 @@
         <v>2009</v>
       </c>
       <c r="B2" t="n">
-        <v>42121.07</v>
+        <v>48049.67</v>
       </c>
       <c r="C2" t="n">
-        <v>468759.85</v>
+        <v>232110.5</v>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -457,13 +457,13 @@
         <v>2010</v>
       </c>
       <c r="B3" t="n">
-        <v>208034.09</v>
+        <v>203491.03</v>
       </c>
       <c r="C3" t="n">
-        <v>2057605.57</v>
+        <v>913901.36</v>
       </c>
       <c r="D3" t="n">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4">
@@ -471,13 +471,13 @@
         <v>2011</v>
       </c>
       <c r="B4" t="n">
-        <v>260917.98</v>
+        <v>235170.65</v>
       </c>
       <c r="C4" t="n">
-        <v>2261342.3</v>
+        <v>959247.12</v>
       </c>
       <c r="D4" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
@@ -485,13 +485,13 @@
         <v>2012</v>
       </c>
       <c r="B5" t="n">
-        <v>197372.39</v>
+        <v>176509.47</v>
       </c>
       <c r="C5" t="n">
-        <v>1482720.67</v>
+        <v>651665.23</v>
       </c>
       <c r="D5" t="n">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -499,13 +499,13 @@
         <v>2013</v>
       </c>
       <c r="B6" t="n">
-        <v>135545.72</v>
+        <v>120182.57</v>
       </c>
       <c r="C6" t="n">
-        <v>882711.75</v>
+        <v>412303.82</v>
       </c>
       <c r="D6" t="n">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7">
@@ -513,13 +513,13 @@
         <v>2014</v>
       </c>
       <c r="B7" t="n">
-        <v>81877.21000000001</v>
+        <v>71805.83</v>
       </c>
       <c r="C7" t="n">
-        <v>462432.6</v>
+        <v>225032.72</v>
       </c>
       <c r="D7" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8">
@@ -527,13 +527,13 @@
         <v>2015</v>
       </c>
       <c r="B8" t="n">
-        <v>43392.84</v>
+        <v>37664.26</v>
       </c>
       <c r="C8" t="n">
-        <v>212470.62</v>
+        <v>105701.41</v>
       </c>
       <c r="D8" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9">
@@ -541,13 +541,13 @@
         <v>2016</v>
       </c>
       <c r="B9" t="n">
-        <v>17526.91</v>
+        <v>14660.65</v>
       </c>
       <c r="C9" t="n">
-        <v>74755.72</v>
+        <v>36340.89</v>
       </c>
       <c r="D9" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
@@ -555,10 +555,10 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>5312.5</v>
+        <v>4325.3</v>
       </c>
       <c r="C10" t="n">
-        <v>19663.97</v>
+        <v>9512.110000000001</v>
       </c>
       <c r="D10" t="n">
         <v>12</v>
@@ -569,13 +569,13 @@
         <v>2018</v>
       </c>
       <c r="B11" t="n">
-        <v>156.25</v>
+        <v>48.06</v>
       </c>
       <c r="C11" t="n">
-        <v>523.52</v>
+        <v>99.77</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ContAgil advanced flow summary (pasta + original + SELIC).
Introduces scripts/resumo_fluxos_avancado.py matching the WinPython CLI:
reads saida/fluxos_*, joins operations Excel, recalculates ContAgil impact
via STP column D, and writes a multi-sheet workbook plus individual resumos.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/impacto_fiscal_por_ano.xlsx
+++ b/output/impacto_fiscal_por_ano.xlsx
@@ -443,13 +443,13 @@
         <v>2009</v>
       </c>
       <c r="B2" t="n">
-        <v>48049.67</v>
+        <v>110576.45</v>
       </c>
       <c r="C2" t="n">
-        <v>232110.5</v>
+        <v>535399.58</v>
       </c>
       <c r="D2" t="n">
-        <v>47</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3">
@@ -457,13 +457,13 @@
         <v>2010</v>
       </c>
       <c r="B3" t="n">
-        <v>203491.03</v>
+        <v>426303.6</v>
       </c>
       <c r="C3" t="n">
-        <v>913901.36</v>
+        <v>1914530.92</v>
       </c>
       <c r="D3" t="n">
-        <v>180</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4">
@@ -471,13 +471,13 @@
         <v>2011</v>
       </c>
       <c r="B4" t="n">
-        <v>235170.65</v>
+        <v>500843.63</v>
       </c>
       <c r="C4" t="n">
-        <v>959247.12</v>
+        <v>2044218.57</v>
       </c>
       <c r="D4" t="n">
-        <v>237</v>
+        <v>711</v>
       </c>
     </row>
     <row r="5">
@@ -485,13 +485,13 @@
         <v>2012</v>
       </c>
       <c r="B5" t="n">
-        <v>176509.47</v>
+        <v>362423.89</v>
       </c>
       <c r="C5" t="n">
-        <v>651665.23</v>
+        <v>1338706.73</v>
       </c>
       <c r="D5" t="n">
-        <v>209</v>
+        <v>627</v>
       </c>
     </row>
     <row r="6">
@@ -499,13 +499,13 @@
         <v>2013</v>
       </c>
       <c r="B6" t="n">
-        <v>120182.57</v>
+        <v>233352.15</v>
       </c>
       <c r="C6" t="n">
-        <v>412303.82</v>
+        <v>801054.4399999999</v>
       </c>
       <c r="D6" t="n">
-        <v>181</v>
+        <v>543</v>
       </c>
     </row>
     <row r="7">
@@ -513,13 +513,13 @@
         <v>2014</v>
       </c>
       <c r="B7" t="n">
-        <v>71805.83</v>
+        <v>128131.15</v>
       </c>
       <c r="C7" t="n">
-        <v>225032.72</v>
+        <v>401984.19</v>
       </c>
       <c r="D7" t="n">
-        <v>125</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8">
@@ -527,13 +527,13 @@
         <v>2015</v>
       </c>
       <c r="B8" t="n">
-        <v>37664.26</v>
+        <v>62205.63</v>
       </c>
       <c r="C8" t="n">
-        <v>105701.41</v>
+        <v>174799.94</v>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
@@ -541,13 +541,13 @@
         <v>2016</v>
       </c>
       <c r="B9" t="n">
-        <v>14660.65</v>
+        <v>21077.66</v>
       </c>
       <c r="C9" t="n">
-        <v>36340.89</v>
+        <v>52390.84</v>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
@@ -555,13 +555,13 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>4325.3</v>
+        <v>5323.52</v>
       </c>
       <c r="C10" t="n">
-        <v>9512.110000000001</v>
+        <v>11710.96</v>
       </c>
       <c r="D10" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -569,13 +569,13 @@
         <v>2018</v>
       </c>
       <c r="B11" t="n">
-        <v>48.06</v>
+        <v>59.15</v>
       </c>
       <c r="C11" t="n">
-        <v>99.77</v>
+        <v>122.83</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>